<commit_message>
update to do list
</commit_message>
<xml_diff>
--- a/todolist.xlsx
+++ b/todolist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaron/Documents/games/scream_jam_game/gj_itchio_21/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97618E2A-DF5B-5741-B4E7-445C41AF31FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B06667-03B3-0742-8138-3F73411E559E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="1320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
   <si>
     <t>Good To Have</t>
   </si>
@@ -39,31 +39,91 @@
     <t>To Do !</t>
   </si>
   <si>
-    <t>Player Controller</t>
-  </si>
-  <si>
-    <t>3d Modelling</t>
-  </si>
-  <si>
     <t>Opening Cutscene</t>
   </si>
   <si>
-    <t>Briefe</t>
-  </si>
-  <si>
-    <t>End Cutscene</t>
-  </si>
-  <si>
-    <t>Monster Design</t>
-  </si>
-  <si>
-    <t>Map Layout</t>
-  </si>
-  <si>
     <t>Sfx</t>
   </si>
   <si>
     <t>Musik</t>
+  </si>
+  <si>
+    <t>Assets:</t>
+  </si>
+  <si>
+    <t>Türen (2-3 Varianten)</t>
+  </si>
+  <si>
+    <t>Stühle</t>
+  </si>
+  <si>
+    <t>Bürosessel</t>
+  </si>
+  <si>
+    <t>Pflanzen (3-4 Varianten)</t>
+  </si>
+  <si>
+    <t>Tische (3-4 Varianten)</t>
+  </si>
+  <si>
+    <t>Bilderrahmen (2 Varianten)</t>
+  </si>
+  <si>
+    <t>Computer</t>
+  </si>
+  <si>
+    <t>Telephon</t>
+  </si>
+  <si>
+    <t>Ordner (2 Variantern)</t>
+  </si>
+  <si>
+    <t>Geländer von Stiegen</t>
+  </si>
+  <si>
+    <t>Deckenlampen (2 Varianten)</t>
+  </si>
+  <si>
+    <t>Stehlampen (2 Varianten)</t>
+  </si>
+  <si>
+    <t>Mülleimer</t>
+  </si>
+  <si>
+    <t>Schränke (2-3 Varianten)</t>
+  </si>
+  <si>
+    <t>Gemälde (4+ Varianten)</t>
+  </si>
+  <si>
+    <t>Aufzug</t>
+  </si>
+  <si>
+    <t>Teppiche (3-4 Varianten)</t>
+  </si>
+  <si>
+    <t>Tobi</t>
+  </si>
+  <si>
+    <t>Aaron</t>
+  </si>
+  <si>
+    <t>Micheal</t>
+  </si>
+  <si>
+    <t>Anderes:</t>
+  </si>
+  <si>
+    <t>Start Screen</t>
+  </si>
+  <si>
+    <t>Zettel</t>
+  </si>
+  <si>
+    <t>Credits</t>
+  </si>
+  <si>
+    <t>E-Mails</t>
   </si>
 </sst>
 </file>
@@ -73,6 +133,13 @@
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,21 +161,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="20"/>
       <color theme="1"/>
@@ -116,8 +168,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -138,13 +195,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -161,19 +224,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,235 +525,315 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
     <row r="3" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="3"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+    </row>
+    <row r="5" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+    </row>
+    <row r="6" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="D6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+    </row>
+    <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="4"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-    </row>
-    <row r="5" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="6"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
-    </row>
-    <row r="6" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-    </row>
-    <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
+      <c r="D7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
     </row>
     <row r="8" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
     </row>
     <row r="9" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
+      <c r="A9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
     </row>
     <row r="10" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
+      <c r="A10" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
     </row>
     <row r="11" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
+      <c r="A11" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
     </row>
     <row r="12" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
+      <c r="A12" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
     </row>
     <row r="13" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
     </row>
     <row r="14" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
+      <c r="A14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
     </row>
     <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="11"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-    </row>
-    <row r="16" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="17" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="18" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="8"/>
-    </row>
-    <row r="20" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="A15" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="8"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+    </row>
+    <row r="16" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
to do list update
</commit_message>
<xml_diff>
--- a/todolist.xlsx
+++ b/todolist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaron/Documents/games/scream_jam_game/gj_itchio_21/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2270C64-14F9-CE4E-84CF-97AF772CA417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCB715DF-08FE-A14C-BD15-EA113BEFD284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="33">
   <si>
     <t>Good To Have</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Geländer von Stiegen</t>
   </si>
   <si>
-    <t>Deckenlampen (2 Varianten)</t>
-  </si>
-  <si>
     <t>Stehlampen (2 Varianten)</t>
   </si>
   <si>
@@ -124,6 +121,9 @@
   </si>
   <si>
     <t>E-Mails (3)</t>
+  </si>
+  <si>
+    <t>Aaron, Tobi</t>
   </si>
 </sst>
 </file>
@@ -174,7 +174,7 @@
       <name val="Calibri (Body)"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -205,6 +205,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -218,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -232,6 +238,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,7 +544,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
@@ -545,10 +552,10 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -556,10 +563,10 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -576,7 +583,7 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>4</v>
@@ -598,13 +605,13 @@
         <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E6" s="7"/>
       <c r="H6" s="7"/>
@@ -616,15 +623,17 @@
       <c r="N6" s="7"/>
     </row>
     <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="1" t="s">
+      <c r="A7" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7" s="7"/>
       <c r="H7" s="7"/>
@@ -640,12 +649,14 @@
         <v>12</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="7"/>
       <c r="E8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
@@ -656,10 +667,12 @@
       <c r="N8" s="7"/>
     </row>
     <row r="9" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="7"/>
+      <c r="A9" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
@@ -677,7 +690,7 @@
         <v>13</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -696,7 +709,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -715,7 +728,7 @@
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -735,7 +748,7 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -751,10 +764,10 @@
       <c r="N13" s="7"/>
     </row>
     <row r="14" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="7"/>
+      <c r="B14" s="8"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
@@ -769,10 +782,12 @@
       <c r="N14" s="7"/>
     </row>
     <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="8"/>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
@@ -787,42 +802,35 @@
       <c r="N15" s="7"/>
     </row>
     <row r="16" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
     <row r="18" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>23</v>
+      <c r="A19" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" t="s">
-        <v>26</v>
-      </c>
-    </row>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="21" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="23" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>